<commit_message>
feat: improve workforce app, auth, employee portal and mobile UI
</commit_message>
<xml_diff>
--- a/backend/test_excel_v2_empty.xlsx
+++ b/backend/test_excel_v2_empty.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Zusammenfassung" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Arbeitszeiten" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Standortauswertung" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Mitarbeiteruebersicht" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zusammenfassung" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Arbeitszeiten" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Standortauswertung" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mitarbeiteruebersicht" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Arbeitszeiten'!$A$1:$H$1</definedName>
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,8 +40,42 @@
       <color rgb="FFFFFFFF"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001E3A5F"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00555555"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -53,8 +87,33 @@
         <fgColor rgb="FF1E3A5F"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001E3A5F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EEF4FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6E8F7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E5F8A"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -62,15 +121,63 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B0C8E0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B0C8E0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B0C8E0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B0C8E0"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -437,150 +544,161 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="27" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="38" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Time Stemple – Monatsbericht</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="6" customHeight="1">
+      <c r="A2" s="4" t="n"/>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>Zeitraum</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>2026-06-01 – 2026-06-30</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Mitarbeiter</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Alle</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr"/>
-      <c r="B3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+    <row r="5" ht="8" customHeight="1"/>
+    <row r="6" ht="26" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>KPI</t>
         </is>
       </c>
-      <c r="B4" s="1" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>Wert</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Gesamtstunden (h)</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>0:00</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Offizielle Stunden (h)</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>0:00</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>Ausstehend (h)</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>0:00</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>Soll-Stunden (h)</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>Differenz (h)</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>0:00</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>Schichten</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>Arbeitstage</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>Standorte</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -591,56 +709,63 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>Arbeitszeiten – Detailansicht</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="13" t="inlineStr">
         <is>
           <t>Datum</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B2" s="13" t="inlineStr">
         <is>
           <t>Wochentag</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C2" s="13" t="inlineStr">
         <is>
           <t>Standort</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D2" s="13" t="inlineStr">
         <is>
           <t>Check-In</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E2" s="13" t="inlineStr">
         <is>
           <t>Check-Out</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F2" s="13" t="inlineStr">
         <is>
           <t>Pause</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G2" s="13" t="inlineStr">
         <is>
           <t>Arbeitszeit</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H2" s="13" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -648,6 +773,9 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -658,41 +786,48 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>Standortauswertung</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="13" t="inlineStr">
         <is>
           <t>Standort</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B2" s="13" t="inlineStr">
         <is>
           <t>Anzahl Schichten</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C2" s="13" t="inlineStr">
         <is>
           <t>Stunden</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>GESAMT</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B3" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C3" s="14" t="inlineStr">
         <is>
           <t>0:00</t>
         </is>
@@ -700,6 +835,9 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:C1"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -710,56 +848,63 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>Mitarbeiterübersicht</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="13" t="inlineStr">
         <is>
           <t>Mitarbeiter</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B2" s="13" t="inlineStr">
         <is>
           <t>E-Mail</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C2" s="13" t="inlineStr">
         <is>
           <t>Offizielle Stunden</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D2" s="13" t="inlineStr">
         <is>
           <t>Ausstehend</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E2" s="13" t="inlineStr">
         <is>
           <t>Schichten</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F2" s="13" t="inlineStr">
         <is>
           <t>Arbeitstage</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G2" s="13" t="inlineStr">
         <is>
           <t>Soll (h)</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H2" s="13" t="inlineStr">
         <is>
           <t>Differenz (h)</t>
         </is>
@@ -767,6 +912,9 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>